<commit_message>
revert the cbm-hwp model back to using timestep instead of year
</commit_message>
<xml_diff>
--- a/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
+++ b/models/demo-cbm-hwp/demo-cbm-hwp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-public-releases/models/demo-cbm-hwp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B946D7-90E6-C943-BA8A-31D537D69FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68BAC573-EB08-2C44-989C-0C72E9EB3EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="32680" windowHeight="21320" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19900" yWindow="1400" windowWidth="28000" windowHeight="25920" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs - Flow Network" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="142">
   <si>
     <t>Keyword: POOL</t>
   </si>
@@ -278,9 +278,6 @@
     <t>Landfill Module ON/OFF Switch</t>
   </si>
   <si>
-    <t>ON</t>
-  </si>
-  <si>
     <t>Aerobic conditions</t>
   </si>
   <si>
@@ -507,13 +504,16 @@
   </si>
   <si>
     <t>Species Rule</t>
+  </si>
+  <si>
+    <t>OFF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -549,6 +549,12 @@
       <name val="HelveticaNeue"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -582,7 +588,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -592,6 +598,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -875,21 +882,6 @@
             <v>26583833.232000001</v>
           </cell>
         </row>
-        <row r="38">
-          <cell r="H38">
-            <v>9100636.3300000001</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="H74">
-            <v>1575533</v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="H110">
-            <v>6458552</v>
-          </cell>
-        </row>
       </sheetData>
     </sheetDataSet>
   </externalBook>
@@ -1096,7 +1088,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="13.140625" style="1" customWidth="1"/>
@@ -1311,7 +1303,7 @@
     <row r="24" spans="1:12" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B24" s="1" t="s">
         <v>33</v>
@@ -1639,7 +1631,7 @@
     <row r="48" spans="1:6" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B48" s="1" t="s">
         <v>48</v>
@@ -1663,7 +1655,7 @@
     <row r="49" spans="1:10" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="str">
         <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
+        <v/>
       </c>
       <c r="B49" s="1" t="s">
         <v>48</v>
@@ -1794,7 +1786,7 @@
       <c r="D58" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E58" s="3" t="s">
+      <c r="E58" s="9" t="s">
         <v>32</v>
       </c>
       <c r="F58" s="2" t="s">
@@ -1812,18 +1804,15 @@
         <v>54</v>
       </c>
       <c r="C60" s="1" t="str">
-        <f>C31 &amp; ", 1990"</f>
-        <v>Manufacturing, 1990</v>
+        <f>C31 &amp; ", 1990-2000"</f>
+        <v>Manufacturing, 1990-2000</v>
       </c>
       <c r="D60" s="1" t="str">
         <f>C31</f>
         <v>Manufacturing</v>
       </c>
-      <c r="E60" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F60" s="1">
-        <v>1990</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="15.75" customHeight="1">
@@ -1831,18 +1820,15 @@
         <v>54</v>
       </c>
       <c r="C61" s="1" t="str">
-        <f>C32 &amp; ", 1991"</f>
-        <v>Manufacturing, 1991</v>
+        <f>C32 &amp; ", 2001-"</f>
+        <v>Manufacturing, 2001-</v>
       </c>
       <c r="D61" s="1" t="str">
         <f>C31</f>
         <v>Manufacturing</v>
       </c>
-      <c r="E61" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="F61" s="1">
-        <v>1991</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" spans="1:10" s="2" customFormat="1" ht="15.75" customHeight="1">
@@ -1859,315 +1845,280 @@
         <v>58</v>
       </c>
       <c r="F63" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>59</v>
       </c>
       <c r="H63" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="I63" s="8" t="s">
         <v>140</v>
-      </c>
-      <c r="I63" s="8" t="s">
-        <v>141</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A65" s="1" t="s">
-        <v>61</v>
-      </c>
+    <row r="65" spans="2:7" ht="15.75" customHeight="1">
       <c r="B65" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C65" s="1" t="str">
-        <f>C60</f>
-        <v>Manufacturing, 1990</v>
+        <f>$C$60</f>
+        <v>Manufacturing, 1990-2000</v>
       </c>
       <c r="D65" s="1">
         <f>F32</f>
         <v>1</v>
       </c>
-      <c r="F65" s="1">
-        <f>[1]Sheet1!$H$38</f>
-        <v>9100636.3300000001</v>
+      <c r="E65" s="1">
+        <v>0.35</v>
       </c>
       <c r="G65" s="1" t="str">
         <f>'Inputs - Tags'!C4</f>
         <v>Sawnwood</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A66" s="1" t="s">
-        <v>61</v>
-      </c>
+    <row r="66" spans="2:7" ht="15.75" customHeight="1">
       <c r="B66" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C66" s="1" t="str">
-        <f>C60</f>
-        <v>Manufacturing, 1990</v>
+        <f>$C$60</f>
+        <v>Manufacturing, 1990-2000</v>
       </c>
       <c r="D66" s="1">
         <f>F33</f>
         <v>2</v>
       </c>
-      <c r="F66" s="1">
-        <f>[1]Sheet1!$H$74</f>
-        <v>1575533</v>
+      <c r="E66" s="1">
+        <v>0.05</v>
       </c>
       <c r="G66" s="1" t="str">
         <f>'Inputs - Tags'!C5</f>
         <v>Panels</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="15.75" customHeight="1">
-      <c r="A67" s="1" t="s">
-        <v>61</v>
-      </c>
+    <row r="67" spans="2:7" ht="15.75" customHeight="1">
       <c r="B67" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C67" s="1" t="str">
-        <f>C60</f>
-        <v>Manufacturing, 1990</v>
+        <f>$C$60</f>
+        <v>Manufacturing, 1990-2000</v>
       </c>
       <c r="D67" s="1">
         <f>F34</f>
         <v>3</v>
       </c>
-      <c r="F67" s="1">
-        <f>[1]Sheet1!$H$110</f>
-        <v>6458552</v>
+      <c r="E67" s="1">
+        <v>0.2</v>
       </c>
       <c r="G67" s="1" t="str">
         <f>'Inputs - Tags'!C6</f>
         <v>Paper</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="15.75" customHeight="1">
-      <c r="B69" s="1" t="s">
+    <row r="68" spans="2:7" ht="15.75" customHeight="1">
+      <c r="B68" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C69" s="1" t="str">
+      <c r="C68" s="1" t="str">
         <f>$C$60</f>
-        <v>Manufacturing, 1990</v>
-      </c>
-      <c r="D69" s="1">
+        <v>Manufacturing, 1990-2000</v>
+      </c>
+      <c r="D68" s="1">
+        <f>F35</f>
+        <v>4</v>
+      </c>
+      <c r="E68" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="G68" s="1" t="str">
+        <f>'Inputs - Tags'!C7</f>
+        <v>Bioenergy</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" ht="15.75" customHeight="1">
+      <c r="B70" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C70" s="1" t="str">
+        <f>$C$61</f>
+        <v>Manufacturing, 2001-</v>
+      </c>
+      <c r="D70" s="1">
         <f>F32</f>
         <v>1</v>
       </c>
-      <c r="E69" s="1">
-        <v>0.35</v>
-      </c>
-      <c r="G69" s="1" t="str">
+      <c r="E70" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="G70" s="1" t="str">
         <f>'Inputs - Tags'!C4</f>
         <v>Sawnwood</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="15.75" customHeight="1">
-      <c r="B70" s="1" t="s">
+    <row r="71" spans="2:7" ht="15.75" customHeight="1">
+      <c r="B71" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C70" s="1" t="str">
-        <f>$C$60</f>
-        <v>Manufacturing, 1990</v>
-      </c>
-      <c r="D70" s="1">
+      <c r="C71" s="1" t="str">
+        <f>$C$61</f>
+        <v>Manufacturing, 2001-</v>
+      </c>
+      <c r="D71" s="1">
         <f>F33</f>
         <v>2</v>
       </c>
-      <c r="E70" s="1">
+      <c r="E71" s="1">
         <v>0.05</v>
       </c>
-      <c r="G70" s="1" t="str">
+      <c r="G71" s="1" t="str">
         <f>'Inputs - Tags'!C5</f>
         <v>Panels</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="15.75" customHeight="1">
-      <c r="B71" s="1" t="s">
+    <row r="72" spans="2:7" ht="15.75" customHeight="1">
+      <c r="B72" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C71" s="1" t="str">
-        <f>$C$60</f>
-        <v>Manufacturing, 1990</v>
-      </c>
-      <c r="D71" s="1">
+      <c r="C72" s="1" t="str">
+        <f>$C$61</f>
+        <v>Manufacturing, 2001-</v>
+      </c>
+      <c r="D72" s="1">
         <f>F34</f>
         <v>3</v>
       </c>
-      <c r="E71" s="1">
-        <v>0.2</v>
-      </c>
-      <c r="G71" s="1" t="str">
+      <c r="E72" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="G72" s="1" t="str">
         <f>'Inputs - Tags'!C6</f>
         <v>Paper</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="15.75" customHeight="1">
-      <c r="B72" s="1" t="s">
+    <row r="73" spans="2:7" ht="15.75" customHeight="1">
+      <c r="B73" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C72" s="1" t="str">
-        <f>$C$60</f>
-        <v>Manufacturing, 1990</v>
-      </c>
-      <c r="D72" s="1">
+      <c r="C73" s="1" t="str">
+        <f>$C$61</f>
+        <v>Manufacturing, 2001-</v>
+      </c>
+      <c r="D73" s="1">
         <f>F35</f>
         <v>4</v>
       </c>
-      <c r="E72" s="1">
-        <v>0.4</v>
-      </c>
-      <c r="G72" s="1" t="str">
+      <c r="E73" s="1">
+        <f>1-SUM(E70:E72)</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="G73" s="1" t="str">
         <f>'Inputs - Tags'!C7</f>
         <v>Bioenergy</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="15.75" customHeight="1">
-      <c r="B74" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C74" s="1" t="str">
-        <f>$C$61</f>
-        <v>Manufacturing, 1991</v>
-      </c>
-      <c r="D74" s="1">
-        <f>F32</f>
-        <v>1</v>
-      </c>
-      <c r="E74" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="G74" s="1" t="str">
-        <f>'Inputs - Tags'!C4</f>
-        <v>Sawnwood</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" ht="15.75" customHeight="1">
+    <row r="75" spans="2:7" ht="15.75" customHeight="1">
       <c r="B75" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C75" s="1" t="str">
-        <f>$C$61</f>
-        <v>Manufacturing, 1991</v>
+        <f>C38</f>
+        <v>Residue Valorizing</v>
       </c>
       <c r="D75" s="1">
-        <f>F33</f>
-        <v>2</v>
+        <f>F38</f>
+        <v>1</v>
       </c>
       <c r="E75" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="G75" s="1" t="str">
-        <f>'Inputs - Tags'!C5</f>
-        <v>Panels</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" ht="15.75" customHeight="1">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" ht="15.75" customHeight="1">
       <c r="B76" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C76" s="1" t="str">
-        <f>$C$61</f>
-        <v>Manufacturing, 1991</v>
+        <f>C39</f>
+        <v>Residue Valorizing</v>
       </c>
       <c r="D76" s="1">
-        <f>F34</f>
-        <v>3</v>
+        <f>F39</f>
+        <v>2</v>
       </c>
       <c r="E76" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="G76" s="1" t="str">
-        <f>'Inputs - Tags'!C6</f>
-        <v>Paper</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" ht="15.75" customHeight="1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" ht="15.75" customHeight="1">
       <c r="B77" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C77" s="1" t="str">
-        <f>$C$61</f>
-        <v>Manufacturing, 1991</v>
+        <f>C40</f>
+        <v>Residue Valorizing</v>
       </c>
       <c r="D77" s="1">
-        <f>F35</f>
-        <v>4</v>
+        <f>F40</f>
+        <v>3</v>
       </c>
       <c r="E77" s="1">
         <v>0</v>
       </c>
-      <c r="G77" s="1" t="str">
-        <f>'Inputs - Tags'!C7</f>
-        <v>Bioenergy</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" ht="15.75" customHeight="1">
+    </row>
+    <row r="79" spans="2:7" ht="15.75" customHeight="1">
       <c r="B79" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C79" s="1" t="str">
-        <f>C38</f>
-        <v>Residue Valorizing</v>
+        <f>C45</f>
+        <v>Post-consumer Processing</v>
       </c>
       <c r="D79" s="1">
-        <f>F38</f>
+        <f>F45</f>
         <v>1</v>
       </c>
       <c r="E79" s="1">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" ht="15.75" customHeight="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" ht="15.75" customHeight="1">
       <c r="B80" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C80" s="1" t="str">
-        <f>C39</f>
-        <v>Residue Valorizing</v>
+        <f>C46</f>
+        <v>Post-consumer Processing</v>
       </c>
       <c r="D80" s="1">
-        <f>F39</f>
+        <f>F46</f>
         <v>2</v>
       </c>
       <c r="E80" s="1">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B81" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" customHeight="1">
+      <c r="A82" s="1" t="str">
+        <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
+        <v/>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C81" s="1" t="str">
-        <f>C40</f>
-        <v>Residue Valorizing</v>
-      </c>
-      <c r="D81" s="1">
-        <f>F40</f>
-        <v>3</v>
-      </c>
-      <c r="E81" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B83" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C83" s="1" t="str">
-        <f>C45</f>
-        <v>Post-consumer Processing</v>
-      </c>
-      <c r="D83" s="1">
-        <f>F45</f>
-        <v>1</v>
-      </c>
-      <c r="E83" s="1">
-        <v>0</v>
+      <c r="C82" s="1" t="str">
+        <f>$C$49</f>
+        <v>Landfilling</v>
+      </c>
+      <c r="D82" s="1">
+        <f>F49</f>
+        <v>1</v>
+      </c>
+      <c r="E82" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5" ht="15.75" customHeight="1">
@@ -2175,66 +2126,30 @@
         <v>62</v>
       </c>
       <c r="C84" s="1" t="str">
-        <f>C46</f>
-        <v>Post-consumer Processing</v>
+        <f>C52</f>
+        <v>Incinerating</v>
       </c>
       <c r="D84" s="1">
-        <f>F46</f>
-        <v>2</v>
+        <f>F52</f>
+        <v>1</v>
       </c>
       <c r="E84" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A86" s="1" t="str">
-        <f>IF('Inputs - Landfill Module'!$C$3="OFF","","COMMENT")</f>
-        <v>COMMENT</v>
-      </c>
       <c r="B86" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C86" s="1" t="str">
-        <f>$C$49</f>
-        <v>Landfilling</v>
-      </c>
-      <c r="D86" s="1">
-        <f>F49</f>
-        <v>1</v>
-      </c>
-      <c r="E86" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B88" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C88" s="1" t="str">
-        <f>C52</f>
-        <v>Incinerating</v>
-      </c>
-      <c r="D88" s="1">
-        <f>F52</f>
-        <v>1</v>
-      </c>
-      <c r="E88" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="15.75" customHeight="1">
-      <c r="B90" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C90" s="1" t="str">
         <f>C56</f>
         <v>Combusting</v>
       </c>
-      <c r="D90" s="1">
+      <c r="D86" s="1">
         <f>F56</f>
         <v>1</v>
       </c>
-      <c r="E90" s="1">
+      <c r="E86" s="1">
         <v>1</v>
       </c>
     </row>
@@ -2279,7 +2194,7 @@
         <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="2" customFormat="1" ht="15.75" customHeight="1">
@@ -2321,73 +2236,73 @@
     <row r="7" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="str">
         <f t="shared" ref="A7:A22" si="0">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A11" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="13" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A13" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E13" s="1" t="str">
         <f>'Inputs - Curves'!C8</f>
@@ -2397,13 +2312,13 @@
     <row r="14" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E14" s="1" t="str">
         <f>'Inputs - Curves'!C9</f>
@@ -2413,79 +2328,79 @@
     <row r="15" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A17" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A18" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A19" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A22" s="1" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1"/>
@@ -2528,109 +2443,109 @@
     <row r="26" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="str">
         <f t="shared" ref="A26:A34" si="1">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:12" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A32" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A33" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A34" s="1" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1"/>
@@ -2667,7 +2582,7 @@
     <row r="40" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A40" s="1" t="str">
         <f t="shared" ref="A40:A75" si="2">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>48</v>
@@ -2691,7 +2606,7 @@
     <row r="41" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>48</v>
@@ -2715,7 +2630,7 @@
     <row r="42" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>48</v>
@@ -2739,13 +2654,13 @@
     <row r="43" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A44" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>48</v>
@@ -2769,7 +2684,7 @@
     <row r="45" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A45" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>48</v>
@@ -2793,7 +2708,7 @@
     <row r="46" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A46" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>48</v>
@@ -2817,13 +2732,13 @@
     <row r="47" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A47" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A48" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>48</v>
@@ -2847,7 +2762,7 @@
     <row r="49" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A49" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>48</v>
@@ -2871,7 +2786,7 @@
     <row r="50" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A50" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>48</v>
@@ -2895,13 +2810,13 @@
     <row r="51" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A51" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="52" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A52" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>48</v>
@@ -2925,7 +2840,7 @@
     <row r="53" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A53" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>48</v>
@@ -2949,7 +2864,7 @@
     <row r="54" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A54" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>48</v>
@@ -2973,7 +2888,7 @@
     <row r="55" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A55" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>48</v>
@@ -2997,13 +2912,13 @@
     <row r="56" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A56" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="57" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A57" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>48</v>
@@ -3027,7 +2942,7 @@
     <row r="58" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A58" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>48</v>
@@ -3051,7 +2966,7 @@
     <row r="59" spans="1:6" s="1" customFormat="1" ht="15.75" customHeight="1">
       <c r="A59" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>48</v>
@@ -3075,7 +2990,7 @@
     <row r="60" spans="1:6">
       <c r="A60" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>48</v>
@@ -3099,14 +3014,14 @@
     <row r="61" spans="1:6">
       <c r="A61" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B61" s="1"/>
     </row>
     <row r="62" spans="1:6">
       <c r="A62" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>48</v>
@@ -3130,7 +3045,7 @@
     <row r="63" spans="1:6">
       <c r="A63" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>48</v>
@@ -3154,7 +3069,7 @@
     <row r="64" spans="1:6">
       <c r="A64" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>48</v>
@@ -3178,13 +3093,13 @@
     <row r="65" spans="1:10">
       <c r="A65" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>48</v>
@@ -3208,7 +3123,7 @@
     <row r="67" spans="1:10">
       <c r="A67" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>48</v>
@@ -3232,7 +3147,7 @@
     <row r="68" spans="1:10">
       <c r="A68" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>48</v>
@@ -3256,14 +3171,14 @@
     <row r="69" spans="1:10">
       <c r="A69" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B69" s="1"/>
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>48</v>
@@ -3287,7 +3202,7 @@
     <row r="71" spans="1:10">
       <c r="A71" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>48</v>
@@ -3311,7 +3226,7 @@
     <row r="72" spans="1:10">
       <c r="A72" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>48</v>
@@ -3335,14 +3250,14 @@
     <row r="73" spans="1:10">
       <c r="A73" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B73" s="1"/>
     </row>
     <row r="74" spans="1:10">
       <c r="A74" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>48</v>
@@ -3366,7 +3281,7 @@
     <row r="75" spans="1:10">
       <c r="A75" s="1" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>48</v>
@@ -3426,16 +3341,16 @@
         <v>58</v>
       </c>
       <c r="F79" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G79" s="8" t="s">
         <v>59</v>
       </c>
       <c r="H79" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="I79" s="8" t="s">
         <v>140</v>
-      </c>
-      <c r="I79" s="8" t="s">
-        <v>141</v>
       </c>
       <c r="J79" s="2" t="s">
         <v>60</v>
@@ -3445,7 +3360,7 @@
     <row r="81" spans="1:10">
       <c r="A81" s="1" t="str">
         <f t="shared" ref="A81:A112" si="3">IF($C$3="ON","","COMMENT")</f>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>62</v>
@@ -3465,7 +3380,7 @@
     <row r="82" spans="1:10">
       <c r="A82" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>62</v>
@@ -3485,14 +3400,14 @@
     <row r="83" spans="1:10">
       <c r="A83" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B83" s="1"/>
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>62</v>
@@ -3516,7 +3431,7 @@
     <row r="85" spans="1:10">
       <c r="A85" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>62</v>
@@ -3540,14 +3455,14 @@
     <row r="86" spans="1:10">
       <c r="A86" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B86" s="1"/>
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>62</v>
@@ -3564,13 +3479,13 @@
         <v>0.5</v>
       </c>
       <c r="J87" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88" spans="1:10">
       <c r="A88" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>62</v>
@@ -3590,14 +3505,14 @@
     <row r="89" spans="1:10">
       <c r="A89" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B89" s="1"/>
     </row>
     <row r="90" spans="1:10">
       <c r="A90" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>62</v>
@@ -3621,7 +3536,7 @@
     <row r="91" spans="1:10">
       <c r="A91" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>62</v>
@@ -3645,7 +3560,7 @@
     <row r="92" spans="1:10">
       <c r="A92" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B92" s="1"/>
       <c r="C92" s="1"/>
@@ -3653,7 +3568,7 @@
     <row r="93" spans="1:10">
       <c r="A93" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>62</v>
@@ -3673,7 +3588,7 @@
     <row r="94" spans="1:10">
       <c r="A94" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>62</v>
@@ -3690,20 +3605,20 @@
         <v>1</v>
       </c>
       <c r="J94" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B95" s="1"/>
     </row>
     <row r="96" spans="1:10">
       <c r="A96" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>62</v>
@@ -3723,7 +3638,7 @@
     <row r="97" spans="1:5">
       <c r="A97" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>62</v>
@@ -3743,14 +3658,14 @@
     <row r="98" spans="1:5">
       <c r="A98" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B98" s="1"/>
     </row>
     <row r="99" spans="1:5">
       <c r="A99" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>62</v>
@@ -3770,7 +3685,7 @@
     <row r="100" spans="1:5">
       <c r="A100" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>62</v>
@@ -3790,7 +3705,7 @@
     <row r="101" spans="1:5">
       <c r="A101" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>62</v>
@@ -3810,14 +3725,14 @@
     <row r="102" spans="1:5">
       <c r="A102" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B102" s="1"/>
     </row>
     <row r="103" spans="1:5">
       <c r="A103" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>62</v>
@@ -3837,7 +3752,7 @@
     <row r="104" spans="1:5">
       <c r="A104" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>62</v>
@@ -3857,13 +3772,13 @@
     <row r="105" spans="1:5">
       <c r="A105" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="A106" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>62</v>
@@ -3883,7 +3798,7 @@
     <row r="107" spans="1:5">
       <c r="A107" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>62</v>
@@ -3903,13 +3818,13 @@
     <row r="108" spans="1:5">
       <c r="A108" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="A109" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>62</v>
@@ -3929,7 +3844,7 @@
     <row r="110" spans="1:5">
       <c r="A110" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>62</v>
@@ -3949,13 +3864,13 @@
     <row r="111" spans="1:5">
       <c r="A111" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="A112" s="1" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>COMMENT</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>62</v>
@@ -4027,31 +3942,31 @@
   <sheetData>
     <row r="1" spans="2:11" s="6" customFormat="1">
       <c r="B1" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="K1" s="6" t="s">
         <v>53</v>
@@ -4059,7 +3974,7 @@
     </row>
     <row r="3" spans="2:11">
       <c r="B3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C3" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4070,12 +3985,15 @@
         <v>37127083</v>
       </c>
       <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="K3">
         <v>1990</v>
       </c>
     </row>
     <row r="4" spans="2:11">
       <c r="B4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C4" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4086,12 +4004,15 @@
         <v>36678472</v>
       </c>
       <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="K4">
         <v>1991</v>
       </c>
     </row>
     <row r="5" spans="2:11">
       <c r="B5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C5" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4102,12 +4023,15 @@
         <v>38905955</v>
       </c>
       <c r="G5">
+        <v>3</v>
+      </c>
+      <c r="K5">
         <v>1992</v>
       </c>
     </row>
     <row r="6" spans="2:11">
       <c r="B6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C6" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4118,12 +4042,15 @@
         <v>40348197</v>
       </c>
       <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="K6">
         <v>1993</v>
       </c>
     </row>
     <row r="7" spans="2:11">
       <c r="B7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C7" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4134,12 +4061,15 @@
         <v>41958296</v>
       </c>
       <c r="G7">
+        <v>5</v>
+      </c>
+      <c r="K7">
         <v>1994</v>
       </c>
     </row>
     <row r="8" spans="2:11">
       <c r="B8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C8" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4150,12 +4080,15 @@
         <v>43150928</v>
       </c>
       <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="K8">
         <v>1995</v>
       </c>
     </row>
     <row r="9" spans="2:11">
       <c r="B9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C9" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4166,12 +4099,15 @@
         <v>43483436</v>
       </c>
       <c r="G9">
+        <v>7</v>
+      </c>
+      <c r="K9">
         <v>1996</v>
       </c>
     </row>
     <row r="10" spans="2:11">
       <c r="B10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C10" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4182,12 +4118,15 @@
         <v>43752282</v>
       </c>
       <c r="G10">
+        <v>8</v>
+      </c>
+      <c r="K10">
         <v>1997</v>
       </c>
     </row>
     <row r="11" spans="2:11">
       <c r="B11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C11" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4198,12 +4137,15 @@
         <v>40519718</v>
       </c>
       <c r="G11">
+        <v>9</v>
+      </c>
+      <c r="K11">
         <v>1998</v>
       </c>
     </row>
     <row r="12" spans="2:11">
       <c r="B12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C12" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4214,12 +4156,15 @@
         <v>44400810</v>
       </c>
       <c r="G12">
+        <v>10</v>
+      </c>
+      <c r="K12">
         <v>1999</v>
       </c>
     </row>
     <row r="13" spans="2:11">
       <c r="B13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C13" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4230,12 +4175,15 @@
         <v>46222505</v>
       </c>
       <c r="G13">
+        <v>11</v>
+      </c>
+      <c r="K13">
         <v>2000</v>
       </c>
     </row>
     <row r="14" spans="2:11">
       <c r="B14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C14" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4246,12 +4194,15 @@
         <v>42560337</v>
       </c>
       <c r="G14">
+        <v>12</v>
+      </c>
+      <c r="K14">
         <v>2001</v>
       </c>
     </row>
     <row r="15" spans="2:11">
       <c r="B15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C15" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4262,12 +4213,15 @@
         <v>45359633</v>
       </c>
       <c r="G15">
+        <v>13</v>
+      </c>
+      <c r="K15">
         <v>2002</v>
       </c>
     </row>
     <row r="16" spans="2:11">
       <c r="B16" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C16" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4278,12 +4232,15 @@
         <v>41138018</v>
       </c>
       <c r="G16">
+        <v>14</v>
+      </c>
+      <c r="K16">
         <v>2003</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:11">
       <c r="B17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C17" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4294,12 +4251,15 @@
         <v>47648717</v>
       </c>
       <c r="G17">
+        <v>15</v>
+      </c>
+      <c r="K17">
         <v>2004</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:11">
       <c r="B18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C18" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4310,12 +4270,15 @@
         <v>46514709</v>
       </c>
       <c r="G18">
+        <v>16</v>
+      </c>
+      <c r="K18">
         <v>2005</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:11">
       <c r="B19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4326,12 +4289,15 @@
         <v>42120199</v>
       </c>
       <c r="G19">
+        <v>17</v>
+      </c>
+      <c r="K19">
         <v>2006</v>
       </c>
     </row>
-    <row r="20" spans="2:7">
+    <row r="20" spans="2:11">
       <c r="B20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C20" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4342,12 +4308,15 @@
         <v>37693171</v>
       </c>
       <c r="G20">
+        <v>18</v>
+      </c>
+      <c r="K20">
         <v>2007</v>
       </c>
     </row>
-    <row r="21" spans="2:7">
+    <row r="21" spans="2:11">
       <c r="B21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C21" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4358,12 +4327,15 @@
         <v>31885044</v>
       </c>
       <c r="G21">
+        <v>19</v>
+      </c>
+      <c r="K21">
         <v>2008</v>
       </c>
     </row>
-    <row r="22" spans="2:7">
+    <row r="22" spans="2:11">
       <c r="B22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C22" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4374,12 +4346,15 @@
         <v>26634074</v>
       </c>
       <c r="G22">
+        <v>20</v>
+      </c>
+      <c r="K22">
         <v>2009</v>
       </c>
     </row>
-    <row r="23" spans="2:7">
+    <row r="23" spans="2:11">
       <c r="B23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C23" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4390,12 +4365,15 @@
         <v>32520977</v>
       </c>
       <c r="G23">
+        <v>21</v>
+      </c>
+      <c r="K23">
         <v>2010</v>
       </c>
     </row>
-    <row r="24" spans="2:7">
+    <row r="24" spans="2:11">
       <c r="B24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C24" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4406,12 +4384,15 @@
         <v>33932796.350000001</v>
       </c>
       <c r="G24">
+        <v>22</v>
+      </c>
+      <c r="K24">
         <v>2011</v>
       </c>
     </row>
-    <row r="25" spans="2:7">
+    <row r="25" spans="2:11">
       <c r="B25" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C25" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4422,12 +4403,15 @@
         <v>33933907</v>
       </c>
       <c r="G25">
+        <v>23</v>
+      </c>
+      <c r="K25">
         <v>2012</v>
       </c>
     </row>
-    <row r="26" spans="2:7">
+    <row r="26" spans="2:11">
       <c r="B26" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C26" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4438,12 +4422,15 @@
         <v>34825414.534000002</v>
       </c>
       <c r="G26">
+        <v>24</v>
+      </c>
+      <c r="K26">
         <v>2013</v>
       </c>
     </row>
-    <row r="27" spans="2:7">
+    <row r="27" spans="2:11">
       <c r="B27" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C27" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4454,12 +4441,15 @@
         <v>35143340.958999999</v>
       </c>
       <c r="G27">
+        <v>25</v>
+      </c>
+      <c r="K27">
         <v>2014</v>
       </c>
     </row>
-    <row r="28" spans="2:7">
+    <row r="28" spans="2:11">
       <c r="B28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C28" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4470,12 +4460,15 @@
         <v>35723207.659999996</v>
       </c>
       <c r="G28">
+        <v>26</v>
+      </c>
+      <c r="K28">
         <v>2015</v>
       </c>
     </row>
-    <row r="29" spans="2:7">
+    <row r="29" spans="2:11">
       <c r="B29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C29" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4486,12 +4479,15 @@
         <v>35894376</v>
       </c>
       <c r="G29">
+        <v>27</v>
+      </c>
+      <c r="K29">
         <v>2016</v>
       </c>
     </row>
-    <row r="30" spans="2:7">
+    <row r="30" spans="2:11">
       <c r="B30" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C30" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4502,12 +4498,15 @@
         <v>35888193</v>
       </c>
       <c r="G30">
+        <v>28</v>
+      </c>
+      <c r="K30">
         <v>2017</v>
       </c>
     </row>
-    <row r="31" spans="2:7">
+    <row r="31" spans="2:11">
       <c r="B31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C31" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4518,12 +4517,15 @@
         <v>35907843.947999999</v>
       </c>
       <c r="G31">
+        <v>29</v>
+      </c>
+      <c r="K31">
         <v>2018</v>
       </c>
     </row>
-    <row r="32" spans="2:7">
+    <row r="32" spans="2:11">
       <c r="B32" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C32" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4534,12 +4536,15 @@
         <v>32447111.447000001</v>
       </c>
       <c r="G32">
+        <v>30</v>
+      </c>
+      <c r="K32">
         <v>2019</v>
       </c>
     </row>
-    <row r="33" spans="2:7">
+    <row r="33" spans="2:11">
       <c r="B33" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C33" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4550,12 +4555,15 @@
         <v>32663199.739999998</v>
       </c>
       <c r="G33">
+        <v>31</v>
+      </c>
+      <c r="K33">
         <v>2020</v>
       </c>
     </row>
-    <row r="34" spans="2:7">
+    <row r="34" spans="2:11">
       <c r="B34" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C34" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4566,12 +4574,15 @@
         <v>33352126.546</v>
       </c>
       <c r="G34">
+        <v>32</v>
+      </c>
+      <c r="K34">
         <v>2021</v>
       </c>
     </row>
-    <row r="35" spans="2:7">
+    <row r="35" spans="2:11">
       <c r="B35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C35" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4582,12 +4593,15 @@
         <v>33352126.546</v>
       </c>
       <c r="G35">
+        <v>33</v>
+      </c>
+      <c r="K35">
         <v>2022</v>
       </c>
     </row>
-    <row r="36" spans="2:7">
+    <row r="36" spans="2:11">
       <c r="B36" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C36" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4598,12 +4612,15 @@
         <v>26583833.232000001</v>
       </c>
       <c r="G36">
+        <v>34</v>
+      </c>
+      <c r="K36">
         <v>2023</v>
       </c>
     </row>
-    <row r="37" spans="2:7">
+    <row r="37" spans="2:11">
       <c r="B37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C37" t="str">
         <f>'Inputs - Flow Network'!$C$3</f>
@@ -4614,6 +4631,9 @@
         <v>26583833.232000001</v>
       </c>
       <c r="G37">
+        <v>35</v>
+      </c>
+      <c r="K37">
         <v>2024</v>
       </c>
     </row>
@@ -4634,18 +4654,18 @@
   <sheetData>
     <row r="1" spans="2:5" s="6" customFormat="1">
       <c r="B1" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -4653,7 +4673,7 @@
     </row>
     <row r="4" spans="2:5">
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
@@ -4661,7 +4681,7 @@
     </row>
     <row r="5" spans="2:5">
       <c r="B5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
@@ -4669,7 +4689,7 @@
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
         <v>17</v>
@@ -4677,15 +4697,15 @@
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
         <v>100</v>
-      </c>
-      <c r="C7" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" spans="2:5" s="6" customFormat="1">
       <c r="B9" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>1</v>
@@ -4699,34 +4719,34 @@
     </row>
     <row r="11" spans="2:5">
       <c r="B11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" t="s">
         <v>103</v>
-      </c>
-      <c r="C11" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="2:5" s="6" customFormat="1">
       <c r="B14" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="D14" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C16" t="str">
         <f>C11</f>
@@ -4739,7 +4759,7 @@
     </row>
     <row r="17" spans="2:7">
       <c r="B17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C17" t="str">
         <f>C11</f>
@@ -4752,7 +4772,7 @@
     </row>
     <row r="19" spans="2:7">
       <c r="B19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C19" t="str">
         <f>C12</f>
@@ -4765,16 +4785,16 @@
     </row>
     <row r="21" spans="2:7" s="6" customFormat="1">
       <c r="B21" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="F21" s="6" t="s">
         <v>52</v>
@@ -4785,7 +4805,7 @@
     </row>
     <row r="23" spans="2:7" s="6" customFormat="1">
       <c r="B23" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>1</v>
@@ -4799,24 +4819,24 @@
     </row>
     <row r="25" spans="2:7" s="6" customFormat="1">
       <c r="B25" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="D25" s="7" t="s">
         <v>115</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="27" spans="2:7" s="6" customFormat="1">
       <c r="B27" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="E27" s="6" t="s">
         <v>53</v>
@@ -4842,13 +4862,13 @@
   <sheetData>
     <row r="1" spans="2:6" s="6" customFormat="1">
       <c r="B1" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>52</v>
@@ -4859,29 +4879,29 @@
     </row>
     <row r="3" spans="2:6">
       <c r="B3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" t="s">
         <v>121</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>122</v>
-      </c>
-      <c r="F3" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="4" spans="2:6">
       <c r="B4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" t="s">
         <v>124</v>
-      </c>
-      <c r="F4" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="6" spans="2:6" s="6" customFormat="1">
       <c r="B6" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>1</v>
@@ -4895,40 +4915,40 @@
     </row>
     <row r="8" spans="2:6">
       <c r="B8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" t="s">
         <v>127</v>
-      </c>
-      <c r="C8" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="9" spans="2:6">
       <c r="B9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="2:6" s="6" customFormat="1">
       <c r="B11" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>131</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>132</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="2:6">
       <c r="B13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C13" t="str">
         <f>C8</f>
@@ -4947,7 +4967,7 @@
     </row>
     <row r="14" spans="2:6">
       <c r="B14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C14" t="str">
         <f>C9</f>
@@ -4966,21 +4986,21 @@
     </row>
     <row r="16" spans="2:6" s="6" customFormat="1">
       <c r="B16" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" t="str">
         <f>$C$3</f>
@@ -4995,7 +5015,7 @@
     </row>
     <row r="19" spans="2:5">
       <c r="B19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C19" t="str">
         <f>$C$3</f>
@@ -5011,7 +5031,7 @@
     </row>
     <row r="21" spans="2:5">
       <c r="B21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C21" t="str">
         <f>C4</f>
@@ -5026,7 +5046,7 @@
     </row>
     <row r="22" spans="2:5">
       <c r="B22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C22" t="str">
         <f>C4</f>

</xml_diff>